<commit_message>
costo puente de grua
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH_costos_nuevos/Costo_fijo/Swap_fixed_3estaciones_320kW/elmo_data.xlsx
+++ b/data/Escenarios_DCH_costos_nuevos/Costo_fijo/Swap_fixed_3estaciones_320kW/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH_costos_nuevos\Costo_fijo\Swap_fixed_3estaciones_320kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FAA932-360F-42F4-ADD8-930771A22395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFFD2A8-D9AB-4BD6-B7AF-459F7D278924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1093" uniqueCount="398">
   <si>
     <t>id</t>
   </si>
@@ -1228,6 +1228,9 @@
   </si>
   <si>
     <t>max_batteries_per_bay</t>
+  </si>
+  <si>
+    <t>c_crane</t>
   </si>
 </sst>
 </file>
@@ -3484,20 +3487,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
-    <col min="8" max="8" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3511,31 +3514,34 @@
         <v>391</v>
       </c>
       <c r="E1" t="s">
+        <v>397</v>
+      </c>
+      <c r="F1" t="s">
         <v>392</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>393</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>394</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>396</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>395</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>373</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>374</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3555,7 +3561,7 @@
         <v>375</v>
       </c>
       <c r="G2" t="s">
-        <v>51</v>
+        <v>375</v>
       </c>
       <c r="H2" t="s">
         <v>51</v>
@@ -3564,16 +3570,19 @@
         <v>51</v>
       </c>
       <c r="J2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" t="s">
         <v>10</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>376</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -3587,13 +3596,13 @@
         <v>38221</v>
       </c>
       <c r="E3">
+        <v>16752</v>
+      </c>
+      <c r="F3">
         <v>5733</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>4389</v>
-      </c>
-      <c r="G3">
-        <v>2</v>
       </c>
       <c r="H3">
         <v>2</v>
@@ -3602,16 +3611,19 @@
         <v>2</v>
       </c>
       <c r="J3">
+        <v>2</v>
+      </c>
+      <c r="K3">
         <v>168</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
       <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -3625,13 +3637,13 @@
         <v>38221</v>
       </c>
       <c r="E4">
+        <v>16752</v>
+      </c>
+      <c r="F4">
         <v>5733</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>4389</v>
-      </c>
-      <c r="G4">
-        <v>2</v>
       </c>
       <c r="H4">
         <v>2</v>
@@ -3640,16 +3652,19 @@
         <v>2</v>
       </c>
       <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
         <v>168</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
       <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>1500</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -3663,13 +3678,13 @@
         <v>38221</v>
       </c>
       <c r="E5">
+        <v>16752</v>
+      </c>
+      <c r="F5">
         <v>5733</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>4389</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
       </c>
       <c r="H5">
         <v>2</v>
@@ -3678,12 +3693,15 @@
         <v>2</v>
       </c>
       <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
         <v>253</v>
       </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
       <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
         <v>1500</v>
       </c>
     </row>

</xml_diff>